<commit_message>
Updated use cases and modified SRS
</commit_message>
<xml_diff>
--- a/Diagramas de casos de uso/Diagramas de casos de uso/Tablas descripcion caso de uso.xlsx
+++ b/Diagramas de casos de uso/Diagramas de casos de uso/Tablas descripcion caso de uso.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="50">
   <si>
     <t>RF1</t>
   </si>
@@ -55,6 +55,9 @@
     <t>Envía un enlace seguro para restablecer la contraseña y confirma el proceso.</t>
   </si>
   <si>
+    <t>El sistema envia una pestaña para que usuario acepte terminos, condiciones y permisos, para el uso del sistema.</t>
+  </si>
+  <si>
     <t>RF2</t>
   </si>
   <si>
@@ -125,6 +128,39 @@
   </si>
   <si>
     <t>Visualiza las alertas y recomendaciones y las marca como revisadas.</t>
+  </si>
+  <si>
+    <t>RF5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Descripción </t>
+  </si>
+  <si>
+    <t>Registra o vincula el dispositivo al sistema</t>
+  </si>
+  <si>
+    <t>Valida las credenciales del dispositivo.</t>
+  </si>
+  <si>
+    <t>Asocia el dispositivo a un proyecto.</t>
+  </si>
+  <si>
+    <t>Envía automáticamente los datos de consumo (voltaje, corriente, potencia, energía) cada 60 segundos.</t>
+  </si>
+  <si>
+    <t>Recibe, valida y almacena los datos en la base de datos.</t>
+  </si>
+  <si>
+    <t>Analiza la última medición para determinar el estado del dispositivo (en línea).</t>
+  </si>
+  <si>
+    <t>Si no recibe datos en el tiempo esperado, marca el dispositivo como fuera de línea.</t>
+  </si>
+  <si>
+    <t>Detecta pérdida de conexión e intenta reconectarse automáticamente.</t>
+  </si>
+  <si>
+    <t>Restablece la conexión y continúa el monitoreo.</t>
   </si>
 </sst>
 </file>
@@ -518,14 +554,20 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="1" t="s">
+    <row r="11">
+      <c r="A11" s="3">
+        <v>9.0</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="s">
-        <v>1</v>
+      <c r="A14" s="1" t="s">
+        <v>15</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>2</v>
@@ -535,79 +577,77 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3">
-        <v>1.0</v>
+      <c r="A15" s="2" t="s">
+        <v>1</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3">
-        <v>5.0</v>
+        <v>4.0</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3">
-        <v>6.0</v>
+        <v>5.0</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="s">
         <v>21</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="1"/>
+    </row>
     <row r="24">
-      <c r="A24" s="2" t="s">
-        <v>1</v>
+      <c r="A24" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>2</v>
@@ -617,79 +657,77 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3">
-        <v>1.0</v>
+      <c r="A25" s="2" t="s">
+        <v>1</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3">
-        <v>5.0</v>
+        <v>4.0</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3">
-        <v>6.0</v>
+        <v>5.0</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="1" t="s">
         <v>28</v>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="1"/>
+    </row>
     <row r="34">
-      <c r="A34" s="2" t="s">
-        <v>1</v>
+      <c r="A34" s="3" t="s">
+        <v>29</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>2</v>
@@ -699,122 +737,212 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="3">
-        <v>1.0</v>
+      <c r="A35" s="2" t="s">
+        <v>1</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3">
-        <v>5.0</v>
+        <v>4.0</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3">
-        <v>6.0</v>
+        <v>5.0</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3">
-        <v>7.0</v>
+        <v>6.0</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3">
-        <v>8.0</v>
+        <v>7.0</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="4"/>
+      <c r="A43" s="1"/>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
     </row>
     <row r="44">
-      <c r="A44" s="1"/>
+      <c r="A44" s="4"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
     </row>
     <row r="45">
-      <c r="A45" s="1"/>
-      <c r="B45" s="1"/>
-      <c r="C45" s="1"/>
+      <c r="A45" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="1"/>
-      <c r="B46" s="1"/>
-      <c r="C46" s="1"/>
+      <c r="A46" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="1"/>
-      <c r="B47" s="1"/>
-      <c r="C47" s="1"/>
+      <c r="A47" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="1"/>
-      <c r="B48" s="1"/>
-      <c r="C48" s="1"/>
+      <c r="A48" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3">
+        <v>6.0</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3">
+        <v>7.0</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3">
+        <v>9.0</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>49</v>
+      </c>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>